<commit_message>
WIP: L0 finish items 1-2 (51904 skeleton assertion, week2 S004 05 Oct rows); not built yet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests-dotnet/fixtures/service-interim/week2/Service Centre till 05 oct 2026/S004_TenderCollectionDetailed.xlsx
+++ b/tests-dotnet/fixtures/service-interim/week2/Service Centre till 05 oct 2026/S004_TenderCollectionDetailed.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -927,6 +927,153 @@
       </c>
       <c r="M10" t="n">
         <v>3200</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BIAW330SYN0010</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AW330</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SAMPLE</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>400</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BIAW330SYN0011</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>AW330</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SAMPLE</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BIAW330SYN0012</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>AW330</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SAMPLE</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>125</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>